<commit_message>
Retest all DLP payload files
</commit_message>
<xml_diff>
--- a/dlp_test/SA_DLP_Test_Data.xlsx
+++ b/dlp_test/SA_DLP_Test_Data.xlsx
@@ -2676,6 +2676,10 @@
 </worksheet>
 </file>
 
+<file path=dlp_retest_marker.txt>DLP retest all-files marker 2026-06-24T161025
+
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{8d2d19fe-994f-45fd-afd4-59964c366a92}" enabled="1" method="Privileged" siteId="{43b173f2-351a-41f2-a03e-f2af81953f59}" contentBits="0" removed="0"/>

</xml_diff>